<commit_message>
Standardize Lu risk-of-bias source provenance
</commit_message>
<xml_diff>
--- a/risk_of_bias.xlsx
+++ b/risk_of_bias.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="3" r:id="R05071dbb47564415"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="6" r:id="Rd0835e727b6b45e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="3" r:id="R8d26734e9a254bab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="6" r:id="R2bc258d788094b6d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2577,7 +2577,7 @@
         <x:v>Randomized crossover order stated; sequence-generation method, simple/block/stratified randomization and concealment not described.</x:v>
       </x:c>
       <x:c r="I72" s="1" t="str">
-        <x:v>Lu 2022; pp3-8, Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3; ROBUST-RCT manual March 2025</x:v>
+        <x:v>PDF pp3–8; Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3</x:v>
       </x:c>
     </x:row>
     <x:row r="73" ht="34" customHeight="1">
@@ -2606,7 +2606,7 @@
         <x:v>Open-label feeding study; concealment procedure not reported.</x:v>
       </x:c>
       <x:c r="I73" s="1" t="str">
-        <x:v>Lu 2022; pp3-8, Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3; ROBUST-RCT manual March 2025</x:v>
+        <x:v>PDF pp3–8; Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3</x:v>
       </x:c>
     </x:row>
     <x:row r="74" ht="34" customHeight="1">
@@ -2635,7 +2635,7 @@
         <x:v>Unblinded timing; matched prepared meals and controlled test-day intake make expectation-related differences unlikely.</x:v>
       </x:c>
       <x:c r="I74" s="1" t="str">
-        <x:v>Lu 2022; pp3-8, Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3; ROBUST-RCT manual March 2025</x:v>
+        <x:v>PDF pp3–8; Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3</x:v>
       </x:c>
     </x:row>
     <x:row r="75" ht="34" customHeight="1">
@@ -2664,7 +2664,7 @@
         <x:v>Unblinded delivery, but foods were weighed and protocols standardized across the no-preload conditions.</x:v>
       </x:c>
       <x:c r="I75" s="1" t="str">
-        <x:v>Lu 2022; pp3-8, Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3; ROBUST-RCT manual March 2025</x:v>
+        <x:v>PDF pp3–8; Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3</x:v>
       </x:c>
     </x:row>
     <x:row r="76" ht="34" customHeight="1">
@@ -2693,7 +2693,7 @@
         <x:v>Assessor masking not reported; glucose measured instrumentally, limiting judgment. AUC-window reporting ambiguity is recorded separately.</x:v>
       </x:c>
       <x:c r="I76" s="1" t="str">
-        <x:v>Lu 2022; pp3-8, Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3; ROBUST-RCT manual March 2025</x:v>
+        <x:v>PDF pp3–8; Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3</x:v>
       </x:c>
     </x:row>
     <x:row r="77" ht="34" customHeight="1">
@@ -2722,7 +2722,7 @@
         <x:v>All 26 completed CGM. Capillary glucose/insulin absent in 6/26 (23.1%) owing to blood-collection difficulty. Definitely high for capillary outcomes under review thresholds; CGM missing-participant risk definitely low (0/26).</x:v>
       </x:c>
       <x:c r="I77" s="1" t="str">
-        <x:v>Lu 2022; pp3-8, Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3; ROBUST-RCT manual March 2025</x:v>
+        <x:v>PDF pp3–8; Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="34" customHeight="1">
@@ -2751,7 +2751,7 @@
         <x:v>AUC labels describe 0-120 min while methods/curves show -30 to +90; CGM 270-min lunch window overlaps dinner in late condition. Registry cited but not independently verified; endpoint reporting remains uncertain.</x:v>
       </x:c>
       <x:c r="I78" s="1" t="str">
-        <x:v>Lu 2022; pp3-8, Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3; ROBUST-RCT manual March 2025</x:v>
+        <x:v>PDF pp3–8; Methods 2.2/2.5/2.6, Results 3.1/3.3 and Figure 3</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="34" customHeight="1">
@@ -3989,7 +3989,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0972edf215b84b23"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fc67c9a239a427b"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Complete outcome extraction and reconcile source-reported data
</commit_message>
<xml_diff>
--- a/risk_of_bias.xlsx
+++ b/risk_of_bias.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="3" r:id="R8d26734e9a254bab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="6" r:id="R2bc258d788094b6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assessments" sheetId="3" r:id="R1a99ef651d7d4660"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="6" r:id="Ra97bb78fb74449fc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1292,16 +1292,16 @@
         <x:v>Outcome data not included in analysis</x:v>
       </x:c>
       <x:c r="F28" s="1" t="str">
-        <x:v>0/13</x:v>
+        <x:v>1/14 (7.1%)</x:v>
       </x:c>
       <x:c r="G28" s="1" t="str">
-        <x:v>Definitely Low</x:v>
+        <x:v>Probably Low</x:v>
       </x:c>
       <x:c r="H28" s="1" t="str">
-        <x:v>All 13 participants completed both conditions and the entire protocol.</x:v>
+        <x:v>Fourteen participants completed both conditions; one was excluded from analysis for sleep onset latency &gt;60 min, leaving 13 analyzed (7.1% not analyzed).</x:v>
       </x:c>
       <x:c r="I28" s="1" t="str">
-        <x:v>PDF pp3–6; Methods/Tables 2–3</x:v>
+        <x:v>PDF p5; Results, participant flow</x:v>
       </x:c>
     </x:row>
     <x:row r="29" ht="34" customHeight="1">
@@ -3989,7 +3989,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2fc67c9a239a427b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4c4a85603166442d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -4058,7 +4058,7 @@
       </x:c>
       <x:c r="G2" s="6" t="n">
         <x:f>COUNTIFS(Assessments!$D$2:$D$120,6,Assessments!$G$2:$G$120,$A2)</x:f>
-        <x:v>12</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="H2" s="6" t="n">
         <x:f>COUNTIFS(Assessments!$D$2:$D$120,7,Assessments!$G$2:$G$120,$A2)</x:f>
@@ -4095,7 +4095,7 @@
       </x:c>
       <x:c r="G3" s="6" t="n">
         <x:f>COUNTIFS(Assessments!$D$2:$D$120,6,Assessments!$G$2:$G$120,$A3)</x:f>
-        <x:v>0</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="H3" s="6" t="n">
         <x:f>COUNTIFS(Assessments!$D$2:$D$120,7,Assessments!$G$2:$G$120,$A3)</x:f>

</xml_diff>